<commit_message>
Migrate FAQ topic pages: cards-questions block, shared help fragment
New cards-questions block (stacked question link tiles). Importer: faq
template (38 topic pages), cards-questions and fragment parsers, a separate
import script for the shared Still need help? fragment, cleanup for the
topic title/back link, and a migrated-paths map in the links transformer so
links to migrated pages stay on the new site. Fragment block falls back to
/content<path> for local preview.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-planning-tools.report.xlsx
+++ b/tools/importer/reports/import-planning-tools.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="253">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,12 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>error</t>
+  </si>
+  <si>
+    <t>errorStack</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -43,6 +49,9 @@
     <t>["carousel-hero","carousel-hero","cards-service","cards-explore","hero-banner"]</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>index</t>
   </si>
   <si>
@@ -133,6 +142,24 @@
     <t>https://www.toyotafinancial.com/us/en/about_us/company_overview.html</t>
   </si>
   <si>
+    <t>us/en/fragments/faq-help.report.json</t>
+  </si>
+  <si>
+    <t>us/en/fragments/faq-help</t>
+  </si>
+  <si>
+    <t>faq-help-fragment</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:50:52.365Z</t>
+  </si>
+  <si>
+    <t>FAQ help fragment</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/Guaranteed_Auto_Protection_GAP.html</t>
+  </si>
+  <si>
     <t>us/en/planning-tools/faq.report.json</t>
   </si>
   <si>
@@ -145,13 +172,610 @@
     <t>planning-tools</t>
   </si>
   <si>
-    <t>2026-10-03T23:10:29.340Z</t>
+    <t>2026-10-03T23:56:53.371Z</t>
   </si>
   <si>
     <t>FAQs | Toyota Financial</t>
   </si>
   <si>
     <t>https://www.toyotafinancial.com/us/en/planning_tools/faq.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/about-credit.report.json</t>
+  </si>
+  <si>
+    <t>["cards-questions","fragment"]</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/about-credit</t>
+  </si>
+  <si>
+    <t>faq</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:51:29.997Z</t>
+  </si>
+  <si>
+    <t>About Credit | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/about_credit.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/about-tfs.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/about-tfs</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:51:36.310Z</t>
+  </si>
+  <si>
+    <t>About TFS | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/about-tfs.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/about-this-website.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/about-this-website</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:51:42.601Z</t>
+  </si>
+  <si>
+    <t>About this Website | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/about_this_website.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/account-access-and-password.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/account-access-and-password</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:51:47.686Z</t>
+  </si>
+  <si>
+    <t>Account Access and Password | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/account_access_and_password.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/account-details.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/account-details</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:51:53.154Z</t>
+  </si>
+  <si>
+    <t>Account Details | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/account_details.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/account-registration.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/account-registration</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:51:58.343Z</t>
+  </si>
+  <si>
+    <t>Account Registration | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/account_registration.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/billing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/billing</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:02.666Z</t>
+  </si>
+  <si>
+    <t>Billing | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/billing.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/business-solutions.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/business-solutions</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:08.098Z</t>
+  </si>
+  <si>
+    <t>Business Solutions | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/business_solutions.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/bz4x.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/bz4x</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:14.067Z</t>
+  </si>
+  <si>
+    <t>bZ4X | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/bZ4X.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/consent-to-electronic-communications-and-agreements.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/consent-to-electronic-communications-and-agreements</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:19.083Z</t>
+  </si>
+  <si>
+    <t>Consent to Electronic Communications and Agreements | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/consent_to_electronic_communications_and_agreements.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/encrypted-email.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/encrypted-email</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:24.128Z</t>
+  </si>
+  <si>
+    <t>Encrypted Email | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/encrypted-email.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/enrolling-in-pay-online.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/enrolling-in-pay-online</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:29.210Z</t>
+  </si>
+  <si>
+    <t>Enrolling in Pay Online | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/enrolling_in_pay_online.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/extension-and-deferral.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/extension-and-deferral</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:33.522Z</t>
+  </si>
+  <si>
+    <t>Extension and Deferral | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/extension_and_deferral.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/financial-hardship.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/financial-hardship</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:39.616Z</t>
+  </si>
+  <si>
+    <t>Financial Hardship | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/financial-hardship.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/financing-and-protection-products.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/financing-and-protection-products</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:54:35.448Z</t>
+  </si>
+  <si>
+    <t>Vehicle Service Agreements | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/financing_and_protection_products.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/fingerprint-authentication.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/fingerprint-authentication</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:46.031Z</t>
+  </si>
+  <si>
+    <t>Fingerprint Authentication | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/fingerprint_authentication.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/guaranteed-auto-protection-gap.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/guaranteed-auto-protection-gap</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:51.687Z</t>
+  </si>
+  <si>
+    <t>Guaranteed Auto Protection (GAP) | Toyota Financial</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/insurance-in-case-of-accident.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/insurance-in-case-of-accident</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:52:55.599Z</t>
+  </si>
+  <si>
+    <t>Insurance (in case of accident) | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/insurance_in_case_of_accident.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/insurance-requirements.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/insurance-requirements</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:01.023Z</t>
+  </si>
+  <si>
+    <t>Insurance Requirements | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/insurance_requirements.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/lease-end-process.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/lease-end-process</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:07.629Z</t>
+  </si>
+  <si>
+    <t>Lease-End Process | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/lease_end_process.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/loan-payoff-and-title-lien-release.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/loan-payoff-and-title-lien-release</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:13.203Z</t>
+  </si>
+  <si>
+    <t>Loan Payoff and Title/Lien Release | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/loan_payoff_and_title_lien_release.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/login-faqs.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/login-faqs</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:19.409Z</t>
+  </si>
+  <si>
+    <t>Login FAQs | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/login-faqs.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/managing-pay-online.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/managing-pay-online</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:24.500Z</t>
+  </si>
+  <si>
+    <t>Managing Pay Online | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/managing_pay_online.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/marketing-preferences.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/marketing-preferences</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:30.447Z</t>
+  </si>
+  <si>
+    <t>Marketing Preferences | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/marketing_preferences.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/mileage.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/mileage</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:35.773Z</t>
+  </si>
+  <si>
+    <t>Mileage | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/mileage.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/military-benefits.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/military-benefits</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:40.798Z</t>
+  </si>
+  <si>
+    <t>Military Benefits | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/military_benefits.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/mobileapp-faqs.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/mobileapp-faqs</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:45.200Z</t>
+  </si>
+  <si>
+    <t>Mobile app FAQs | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/mobileapp-faqs.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/one-big-beautiful-bill-act.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/one-big-beautiful-bill-act</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:49.874Z</t>
+  </si>
+  <si>
+    <t>One Big Beautiful Bill Act (OBBBA) | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/One_Big_Beautiful_Bill_Act.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/online-credit-application.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/online-credit-application</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:54.147Z</t>
+  </si>
+  <si>
+    <t>Online Credit Application | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/online_credit_application.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/paperless-billing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/paperless-billing</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:53:58.223Z</t>
+  </si>
+  <si>
+    <t>Paperless Billing | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/paperless_billing.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/payments.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/payments</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:54:02.831Z</t>
+  </si>
+  <si>
+    <t>Payments | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/payments.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/privacy.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/privacy</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:54:08.697Z</t>
+  </si>
+  <si>
+    <t>Privacy | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/privacy.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/repeat-customers.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/repeat-customers</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:54:14.842Z</t>
+  </si>
+  <si>
+    <t>Repeat Customers | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/repeat_customers.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/shopping.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/shopping</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:54:20.896Z</t>
+  </si>
+  <si>
+    <t>Shopping | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/shopping.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/support-center.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/support-center</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:54:25.193Z</t>
+  </si>
+  <si>
+    <t>Support Center | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/support_center.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/toyota-insurance.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/toyota-insurance</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:54:30.684Z</t>
+  </si>
+  <si>
+    <t>Toyota Insurance | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/toyota_insurance.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/voluntary-protection-products.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/voluntary-protection-products</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:54:40.225Z</t>
+  </si>
+  <si>
+    <t>Voluntary Protection Products | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/voluntary_protection_products.html</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/wear-and-use.report.json</t>
+  </si>
+  <si>
+    <t>us/en/planning-tools/faq/wear-and-use</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:54:45.160Z</t>
+  </si>
+  <si>
+    <t>Wear and Use | Toyota Financial</t>
+  </si>
+  <si>
+    <t>https://www.toyotafinancial.com/us/en/planning_tools/faq/wear_and_use.html</t>
+  </si>
+  <si>
+    <t>us/en/planning_tools/faq/about_credit.html.report.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: Cannot read properties of undefined (reading 'replace')
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: Cannot read properties of undefined (reading 'replace')
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30
+    at processUrl (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:693:31)
+    at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:956:22)</t>
+  </si>
+  <si>
+    <t>us/en/planning_tools/faq/about_credit.html</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>2026-10-03T23:49:41.188Z</t>
   </si>
 </sst>
 </file>
@@ -540,17 +1164,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="8" width="50" customWidth="1"/>
+    <col min="1" max="5" width="50" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -575,155 +1198,191 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
         <v>20</v>
       </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" t="s">
-        <v>26</v>
-      </c>
       <c r="H4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="H5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="I5" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="I6" t="s">
+        <v>41</v>
+      </c>
+      <c r="J6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F7" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G7" t="s">
         <v>45</v>
@@ -731,9 +1390,1295 @@
       <c r="H7" t="s">
         <v>46</v>
       </c>
+      <c r="I7" t="s">
+        <v>47</v>
+      </c>
+      <c r="J7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" t="s">
+        <v>60</v>
+      </c>
+      <c r="I9" t="s">
+        <v>61</v>
+      </c>
+      <c r="J9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" t="s">
+        <v>65</v>
+      </c>
+      <c r="I10" t="s">
+        <v>66</v>
+      </c>
+      <c r="J10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" t="s">
+        <v>71</v>
+      </c>
+      <c r="J11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>59</v>
+      </c>
+      <c r="H12" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12" t="s">
+        <v>76</v>
+      </c>
+      <c r="J12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>59</v>
+      </c>
+      <c r="H13" t="s">
+        <v>80</v>
+      </c>
+      <c r="I13" t="s">
+        <v>81</v>
+      </c>
+      <c r="J13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14" t="s">
+        <v>85</v>
+      </c>
+      <c r="I14" t="s">
+        <v>86</v>
+      </c>
+      <c r="J14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>89</v>
+      </c>
+      <c r="F15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>59</v>
+      </c>
+      <c r="H15" t="s">
+        <v>90</v>
+      </c>
+      <c r="I15" t="s">
+        <v>91</v>
+      </c>
+      <c r="J15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
+        <v>94</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>59</v>
+      </c>
+      <c r="H16" t="s">
+        <v>95</v>
+      </c>
+      <c r="I16" t="s">
+        <v>96</v>
+      </c>
+      <c r="J16" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>99</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>59</v>
+      </c>
+      <c r="H17" t="s">
+        <v>100</v>
+      </c>
+      <c r="I17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J17" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>104</v>
+      </c>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>59</v>
+      </c>
+      <c r="H18" t="s">
+        <v>105</v>
+      </c>
+      <c r="I18" t="s">
+        <v>106</v>
+      </c>
+      <c r="J18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>59</v>
+      </c>
+      <c r="H19" t="s">
+        <v>110</v>
+      </c>
+      <c r="I19" t="s">
+        <v>111</v>
+      </c>
+      <c r="J19" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>114</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>59</v>
+      </c>
+      <c r="H20" t="s">
+        <v>115</v>
+      </c>
+      <c r="I20" t="s">
+        <v>116</v>
+      </c>
+      <c r="J20" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" t="s">
+        <v>119</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>59</v>
+      </c>
+      <c r="H21" t="s">
+        <v>120</v>
+      </c>
+      <c r="I21" t="s">
+        <v>121</v>
+      </c>
+      <c r="J21" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" t="s">
+        <v>124</v>
+      </c>
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>59</v>
+      </c>
+      <c r="H22" t="s">
+        <v>125</v>
+      </c>
+      <c r="I22" t="s">
+        <v>126</v>
+      </c>
+      <c r="J22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>128</v>
+      </c>
+      <c r="B23" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
+        <v>129</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>59</v>
+      </c>
+      <c r="H23" t="s">
+        <v>130</v>
+      </c>
+      <c r="I23" t="s">
+        <v>131</v>
+      </c>
+      <c r="J23" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>134</v>
+      </c>
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>59</v>
+      </c>
+      <c r="H24" t="s">
+        <v>135</v>
+      </c>
+      <c r="I24" t="s">
+        <v>136</v>
+      </c>
+      <c r="J24" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>139</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>59</v>
+      </c>
+      <c r="H25" t="s">
+        <v>140</v>
+      </c>
+      <c r="I25" t="s">
+        <v>141</v>
+      </c>
+      <c r="J25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>142</v>
+      </c>
+      <c r="B26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
+        <v>143</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>59</v>
+      </c>
+      <c r="H26" t="s">
+        <v>144</v>
+      </c>
+      <c r="I26" t="s">
+        <v>145</v>
+      </c>
+      <c r="J26" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>147</v>
+      </c>
+      <c r="B27" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>148</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" t="s">
+        <v>59</v>
+      </c>
+      <c r="H27" t="s">
+        <v>149</v>
+      </c>
+      <c r="I27" t="s">
+        <v>150</v>
+      </c>
+      <c r="J27" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>152</v>
+      </c>
+      <c r="B28" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>59</v>
+      </c>
+      <c r="H28" t="s">
+        <v>154</v>
+      </c>
+      <c r="I28" t="s">
+        <v>155</v>
+      </c>
+      <c r="J28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>157</v>
+      </c>
+      <c r="B29" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
+        <v>158</v>
+      </c>
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>59</v>
+      </c>
+      <c r="H29" t="s">
+        <v>159</v>
+      </c>
+      <c r="I29" t="s">
+        <v>160</v>
+      </c>
+      <c r="J29" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>162</v>
+      </c>
+      <c r="B30" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
+        <v>163</v>
+      </c>
+      <c r="F30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" t="s">
+        <v>59</v>
+      </c>
+      <c r="H30" t="s">
+        <v>164</v>
+      </c>
+      <c r="I30" t="s">
+        <v>165</v>
+      </c>
+      <c r="J30" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>167</v>
+      </c>
+      <c r="B31" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" t="s">
+        <v>168</v>
+      </c>
+      <c r="F31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" t="s">
+        <v>59</v>
+      </c>
+      <c r="H31" t="s">
+        <v>169</v>
+      </c>
+      <c r="I31" t="s">
+        <v>170</v>
+      </c>
+      <c r="J31" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>172</v>
+      </c>
+      <c r="B32" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" t="s">
+        <v>173</v>
+      </c>
+      <c r="F32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>59</v>
+      </c>
+      <c r="H32" t="s">
+        <v>174</v>
+      </c>
+      <c r="I32" t="s">
+        <v>175</v>
+      </c>
+      <c r="J32" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>177</v>
+      </c>
+      <c r="B33" t="s">
+        <v>57</v>
+      </c>
+      <c r="C33" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>178</v>
+      </c>
+      <c r="F33" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" t="s">
+        <v>59</v>
+      </c>
+      <c r="H33" t="s">
+        <v>179</v>
+      </c>
+      <c r="I33" t="s">
+        <v>180</v>
+      </c>
+      <c r="J33" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>182</v>
+      </c>
+      <c r="B34" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" t="s">
+        <v>183</v>
+      </c>
+      <c r="F34" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" t="s">
+        <v>59</v>
+      </c>
+      <c r="H34" t="s">
+        <v>184</v>
+      </c>
+      <c r="I34" t="s">
+        <v>185</v>
+      </c>
+      <c r="J34" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>187</v>
+      </c>
+      <c r="B35" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>188</v>
+      </c>
+      <c r="F35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" t="s">
+        <v>59</v>
+      </c>
+      <c r="H35" t="s">
+        <v>189</v>
+      </c>
+      <c r="I35" t="s">
+        <v>190</v>
+      </c>
+      <c r="J35" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>192</v>
+      </c>
+      <c r="B36" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
+        <v>193</v>
+      </c>
+      <c r="F36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
+        <v>59</v>
+      </c>
+      <c r="H36" t="s">
+        <v>194</v>
+      </c>
+      <c r="I36" t="s">
+        <v>195</v>
+      </c>
+      <c r="J36" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>197</v>
+      </c>
+      <c r="B37" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" t="s">
+        <v>198</v>
+      </c>
+      <c r="F37" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" t="s">
+        <v>59</v>
+      </c>
+      <c r="H37" t="s">
+        <v>199</v>
+      </c>
+      <c r="I37" t="s">
+        <v>200</v>
+      </c>
+      <c r="J37" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>202</v>
+      </c>
+      <c r="B38" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" t="s">
+        <v>203</v>
+      </c>
+      <c r="F38" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" t="s">
+        <v>59</v>
+      </c>
+      <c r="H38" t="s">
+        <v>204</v>
+      </c>
+      <c r="I38" t="s">
+        <v>205</v>
+      </c>
+      <c r="J38" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>207</v>
+      </c>
+      <c r="B39" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" t="s">
+        <v>208</v>
+      </c>
+      <c r="F39" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" t="s">
+        <v>59</v>
+      </c>
+      <c r="H39" t="s">
+        <v>209</v>
+      </c>
+      <c r="I39" t="s">
+        <v>210</v>
+      </c>
+      <c r="J39" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>212</v>
+      </c>
+      <c r="B40" t="s">
+        <v>57</v>
+      </c>
+      <c r="C40" t="s">
+        <v>12</v>
+      </c>
+      <c r="D40" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" t="s">
+        <v>213</v>
+      </c>
+      <c r="F40" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" t="s">
+        <v>59</v>
+      </c>
+      <c r="H40" t="s">
+        <v>214</v>
+      </c>
+      <c r="I40" t="s">
+        <v>215</v>
+      </c>
+      <c r="J40" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>217</v>
+      </c>
+      <c r="B41" t="s">
+        <v>57</v>
+      </c>
+      <c r="C41" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" t="s">
+        <v>218</v>
+      </c>
+      <c r="F41" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" t="s">
+        <v>59</v>
+      </c>
+      <c r="H41" t="s">
+        <v>219</v>
+      </c>
+      <c r="I41" t="s">
+        <v>220</v>
+      </c>
+      <c r="J41" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>222</v>
+      </c>
+      <c r="B42" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" t="s">
+        <v>223</v>
+      </c>
+      <c r="F42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42" t="s">
+        <v>59</v>
+      </c>
+      <c r="H42" t="s">
+        <v>224</v>
+      </c>
+      <c r="I42" t="s">
+        <v>225</v>
+      </c>
+      <c r="J42" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>227</v>
+      </c>
+      <c r="B43" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" t="s">
+        <v>12</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>228</v>
+      </c>
+      <c r="F43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" t="s">
+        <v>59</v>
+      </c>
+      <c r="H43" t="s">
+        <v>229</v>
+      </c>
+      <c r="I43" t="s">
+        <v>230</v>
+      </c>
+      <c r="J43" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>232</v>
+      </c>
+      <c r="B44" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44" t="s">
+        <v>12</v>
+      </c>
+      <c r="D44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E44" t="s">
+        <v>233</v>
+      </c>
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" t="s">
+        <v>59</v>
+      </c>
+      <c r="H44" t="s">
+        <v>234</v>
+      </c>
+      <c r="I44" t="s">
+        <v>235</v>
+      </c>
+      <c r="J44" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>237</v>
+      </c>
+      <c r="B45" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45" t="s">
+        <v>238</v>
+      </c>
+      <c r="F45" t="s">
+        <v>14</v>
+      </c>
+      <c r="G45" t="s">
+        <v>59</v>
+      </c>
+      <c r="H45" t="s">
+        <v>239</v>
+      </c>
+      <c r="I45" t="s">
+        <v>240</v>
+      </c>
+      <c r="J45" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>242</v>
+      </c>
+      <c r="B46" t="s">
+        <v>57</v>
+      </c>
+      <c r="C46" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E46" t="s">
+        <v>243</v>
+      </c>
+      <c r="F46" t="s">
+        <v>14</v>
+      </c>
+      <c r="G46" t="s">
+        <v>59</v>
+      </c>
+      <c r="H46" t="s">
+        <v>244</v>
+      </c>
+      <c r="I46" t="s">
+        <v>245</v>
+      </c>
+      <c r="J46" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>247</v>
+      </c>
+      <c r="B47" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" t="s">
+        <v>248</v>
+      </c>
+      <c r="D47" t="s">
+        <v>249</v>
+      </c>
+      <c r="E47" t="s">
+        <v>250</v>
+      </c>
+      <c r="F47" t="s">
+        <v>251</v>
+      </c>
+      <c r="G47" t="s">
+        <v>12</v>
+      </c>
+      <c r="H47" t="s">
+        <v>252</v>
+      </c>
+      <c r="I47" t="s">
+        <v>12</v>
+      </c>
+      <c r="J47" t="s">
+        <v>62</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>